<commit_message>
Daily NAV update 2026-03-16
</commit_message>
<xml_diff>
--- a/output/nav_changes_2026-03-16.xlsx
+++ b/output/nav_changes_2026-03-16.xlsx
@@ -551,7 +551,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TMX:DYN27550</t>
+          <t>0P0001ROZ4.TO</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -560,22 +560,16 @@
         </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>15.95</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
+        <v>8.8093</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>8.819000000000001</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>-0.0097</v>
+      </c>
+      <c r="G3" s="6" t="n">
+        <v>-0.0011</v>
       </c>
     </row>
     <row r="4">
@@ -1079,8 +1073,8 @@
       <c r="N2" s="6" t="n">
         <v>-0.0003790000000000001</v>
       </c>
-      <c r="O2" s="7" t="n">
-        <v>0</v>
+      <c r="O2" s="6" t="n">
+        <v>-0.0011</v>
       </c>
     </row>
     <row r="3">
@@ -1128,7 +1122,9 @@
       <c r="N3" s="6" t="n">
         <v>-0.00292</v>
       </c>
-      <c r="O3" t="inlineStr"/>
+      <c r="O3" s="6" t="n">
+        <v>-0.001721</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1175,7 +1171,9 @@
       <c r="N4" s="6" t="n">
         <v>-0.003277</v>
       </c>
-      <c r="O4" t="inlineStr"/>
+      <c r="O4" s="6" t="n">
+        <v>-0.000407</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1222,7 +1220,9 @@
       <c r="N5" s="10" t="n">
         <v>0.000285</v>
       </c>
-      <c r="O5" t="inlineStr"/>
+      <c r="O5" s="10" t="n">
+        <v>0.000374</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1269,7 +1269,9 @@
       <c r="N6" s="10" t="n">
         <v>0.0009779999999999999</v>
       </c>
-      <c r="O6" t="inlineStr"/>
+      <c r="O6" s="10" t="n">
+        <v>0.000215</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1316,7 +1318,9 @@
       <c r="N7" s="6" t="n">
         <v>-0.002977</v>
       </c>
-      <c r="O7" t="inlineStr"/>
+      <c r="O7" s="6" t="n">
+        <v>-0.001165</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1363,7 +1367,9 @@
       <c r="N8" s="6" t="n">
         <v>-0.002675</v>
       </c>
-      <c r="O8" t="inlineStr"/>
+      <c r="O8" s="6" t="n">
+        <v>-0.001051</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1410,7 +1416,9 @@
       <c r="N9" s="10" t="n">
         <v>0.0005369999999999999</v>
       </c>
-      <c r="O9" t="inlineStr"/>
+      <c r="O9" s="10" t="n">
+        <v>8.999999999999999e-05</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1457,7 +1465,9 @@
       <c r="N10" s="6" t="n">
         <v>-0.002377</v>
       </c>
-      <c r="O10" t="inlineStr"/>
+      <c r="O10" s="6" t="n">
+        <v>-0.001354</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1504,7 +1514,9 @@
       <c r="N11" s="6" t="n">
         <v>-0.003236</v>
       </c>
-      <c r="O11" t="inlineStr"/>
+      <c r="O11" s="6" t="n">
+        <v>-0.002049</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1551,7 +1563,9 @@
       <c r="N12" s="10" t="n">
         <v>5e-05</v>
       </c>
-      <c r="O12" t="inlineStr"/>
+      <c r="O12" s="10" t="n">
+        <v>0.0008899999999999999</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1598,7 +1612,9 @@
       <c r="N13" s="10" t="n">
         <v>0.0007570000000000001</v>
       </c>
-      <c r="O13" t="inlineStr"/>
+      <c r="O13" s="10" t="n">
+        <v>0.00062</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1645,7 +1661,9 @@
       <c r="N14" s="6" t="n">
         <v>-0.000202</v>
       </c>
-      <c r="O14" t="inlineStr"/>
+      <c r="O14" s="10" t="n">
+        <v>0.000214</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1692,7 +1710,9 @@
       <c r="N15" s="10" t="n">
         <v>4e-05</v>
       </c>
-      <c r="O15" t="inlineStr"/>
+      <c r="O15" s="6" t="n">
+        <v>-0.000169</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1739,7 +1759,9 @@
       <c r="N16" s="10" t="n">
         <v>0.00098</v>
       </c>
-      <c r="O16" t="inlineStr"/>
+      <c r="O16" s="10" t="n">
+        <v>0.0008010000000000001</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1786,7 +1808,9 @@
       <c r="N17" s="10" t="n">
         <v>0.000445</v>
       </c>
-      <c r="O17" t="inlineStr"/>
+      <c r="O17" s="6" t="n">
+        <v>-4.5e-05</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1833,7 +1857,9 @@
       <c r="N18" s="10" t="n">
         <v>1e-05</v>
       </c>
-      <c r="O18" t="inlineStr"/>
+      <c r="O18" s="10" t="n">
+        <v>0.000181</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1880,7 +1906,9 @@
       <c r="N19" s="10" t="n">
         <v>0.000283</v>
       </c>
-      <c r="O19" t="inlineStr"/>
+      <c r="O19" s="6" t="n">
+        <v>-3.4e-05</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1927,7 +1955,9 @@
       <c r="N20" s="10" t="n">
         <v>0.000779</v>
       </c>
-      <c r="O20" t="inlineStr"/>
+      <c r="O20" s="10" t="n">
+        <v>0.00044</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1974,7 +2004,9 @@
       <c r="N21" s="10" t="n">
         <v>0.001012</v>
       </c>
-      <c r="O21" t="inlineStr"/>
+      <c r="O21" s="10" t="n">
+        <v>0.000384</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2021,7 +2053,9 @@
       <c r="N22" s="10" t="n">
         <v>0.002059</v>
       </c>
-      <c r="O22" t="inlineStr"/>
+      <c r="O22" s="10" t="n">
+        <v>0.000723</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2068,7 +2102,9 @@
       <c r="N23" s="10" t="n">
         <v>0.000365</v>
       </c>
-      <c r="O23" t="inlineStr"/>
+      <c r="O23" s="6" t="n">
+        <v>-0.000825</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2115,7 +2151,9 @@
       <c r="N24" s="10" t="n">
         <v>0.001219</v>
       </c>
-      <c r="O24" t="inlineStr"/>
+      <c r="O24" s="10" t="n">
+        <v>0.000746</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2162,7 +2200,9 @@
       <c r="N25" s="6" t="n">
         <v>-0.000163</v>
       </c>
-      <c r="O25" t="inlineStr"/>
+      <c r="O25" s="10" t="n">
+        <v>0.000317</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2209,7 +2249,9 @@
       <c r="N26" s="10" t="n">
         <v>0.000163</v>
       </c>
-      <c r="O26" t="inlineStr"/>
+      <c r="O26" s="10" t="n">
+        <v>0.000396</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2256,7 +2298,9 @@
       <c r="N27" s="10" t="n">
         <v>0.001058</v>
       </c>
-      <c r="O27" t="inlineStr"/>
+      <c r="O27" s="10" t="n">
+        <v>0.000339</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2303,7 +2347,9 @@
       <c r="N28" s="10" t="n">
         <v>0.000122</v>
       </c>
-      <c r="O28" t="inlineStr"/>
+      <c r="O28" s="10" t="n">
+        <v>0.000623</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2350,7 +2396,9 @@
       <c r="N29" s="6" t="n">
         <v>-0.000122</v>
       </c>
-      <c r="O29" t="inlineStr"/>
+      <c r="O29" s="10" t="n">
+        <v>0.00026</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2397,7 +2445,9 @@
       <c r="N30" s="10" t="n">
         <v>0.000376</v>
       </c>
-      <c r="O30" t="inlineStr"/>
+      <c r="O30" s="10" t="n">
+        <v>0.000193</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2444,7 +2494,9 @@
       <c r="N31" s="10" t="n">
         <v>0.000428</v>
       </c>
-      <c r="O31" t="inlineStr"/>
+      <c r="O31" s="10" t="n">
+        <v>0.000136</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2491,7 +2543,9 @@
       <c r="N32" s="6" t="n">
         <v>-0.000204</v>
       </c>
-      <c r="O32" t="inlineStr"/>
+      <c r="O32" s="10" t="n">
+        <v>6.8e-05</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2538,7 +2592,9 @@
       <c r="N33" s="6" t="n">
         <v>-0.000285</v>
       </c>
-      <c r="O33" t="inlineStr"/>
+      <c r="O33" s="10" t="n">
+        <v>0.000159</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2585,7 +2641,9 @@
       <c r="N34" s="6" t="n">
         <v>-0.00126</v>
       </c>
-      <c r="O34" t="inlineStr"/>
+      <c r="O34" s="10" t="n">
+        <v>0.000317</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2632,7 +2690,9 @@
       <c r="N35" s="10" t="n">
         <v>0.001822</v>
       </c>
-      <c r="O35" t="inlineStr"/>
+      <c r="O35" s="10" t="n">
+        <v>0.001158</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2679,7 +2739,9 @@
       <c r="N36" s="6" t="n">
         <v>-0.000326</v>
       </c>
-      <c r="O36" t="inlineStr"/>
+      <c r="O36" s="6" t="n">
+        <v>-0.000272</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2726,7 +2788,9 @@
       <c r="N37" s="10" t="n">
         <v>0.000896</v>
       </c>
-      <c r="O37" t="inlineStr"/>
+      <c r="O37" s="10" t="n">
+        <v>0.000931</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2773,7 +2837,9 @@
       <c r="N38" s="10" t="n">
         <v>0.001336</v>
       </c>
-      <c r="O38" t="inlineStr"/>
+      <c r="O38" s="10" t="n">
+        <v>0.0007729999999999999</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2818,7 +2884,9 @@
       <c r="N39" s="6" t="n">
         <v>-0.002249</v>
       </c>
-      <c r="O39" t="inlineStr"/>
+      <c r="O39" s="6" t="n">
+        <v>-0.0007040000000000001</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2863,7 +2931,9 @@
       <c r="N40" s="6" t="n">
         <v>-0.000478</v>
       </c>
-      <c r="O40" t="inlineStr"/>
+      <c r="O40" s="10" t="n">
+        <v>0.000329</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">

</xml_diff>